<commit_message>
Use real registered product codes in BT/PB import templates
</commit_message>
<xml_diff>
--- a/public/mau-import-bao-cao-tieu-thu.xlsx
+++ b/public/mau-import-bao-cao-tieu-thu.xlsx
@@ -413,7 +413,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>VG1246060108</v>
+        <v>AZ1664430120-SMS-30759</v>
       </c>
       <c r="B2">
         <v>5</v>
@@ -421,7 +421,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>611600080113</v>
+        <v>AZ1664440069-SMS-30705</v>
       </c>
       <c r="B3">
         <v>20</v>

</xml_diff>